<commit_message>
data: Actualización automática de reportes (2026-10-09 10:15)
</commit_message>
<xml_diff>
--- a/administrador/directorio_asesores.xlsx
+++ b/administrador/directorio_asesores.xlsx
@@ -128,10 +128,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
+        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
+        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
+        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -163,10 +163,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
+        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
+        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
+        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -404,7 +404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:G58"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -934,16 +934,22 @@
         <v>46262</v>
       </c>
     </row>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
+    <row r="58">
+      <c r="A58">
+        <v>119447</v>
+      </c>
+      <c r="B58" t="str">
+        <v>LUIS ANTONIO SALAZAR ESPINOSA</v>
+      </c>
+      <c r="C58">
+        <v>46295</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C46"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G57"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G58"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-10-21 11:21)
</commit_message>
<xml_diff>
--- a/administrador/directorio_asesores.xlsx
+++ b/administrador/directorio_asesores.xlsx
@@ -128,10 +128,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
-        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
-        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
-        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
+        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -163,10 +163,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
-        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
-        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
-        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
+        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -934,6 +934,17 @@
         <v>46262</v>
       </c>
     </row>
+    <row r="49">
+      <c r="A49">
+        <v>21615</v>
+      </c>
+      <c r="B49" t="str">
+        <v>SELINA JANET LEMUS MIRAMONTES</v>
+      </c>
+      <c r="C49">
+        <v>44407</v>
+      </c>
+    </row>
     <row r="58">
       <c r="A58">
         <v>119447</v>

</xml_diff>